<commit_message>
rev A2 (rotations corrected after the JLCPCB preview) — 2026-10-02, from rev-a2-endstand (f736024)
</commit_message>
<xml_diff>
--- a/fertigung/pcbway/BOM_PCBWay.xlsx
+++ b/fertigung/pcbway/BOM_PCBWay.xlsx
@@ -2285,12 +2285,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>LIZ Elec</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>0402WGF6800TCE</t>
+          <t>CR0402FF6800G</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>C25130</t>
+          <t>C100510</t>
         </is>
       </c>
     </row>

</xml_diff>